<commit_message>
20260929_account 전환용 작업 정리
</commit_message>
<xml_diff>
--- a/30_output_share/04_컬럼계보매핑.xlsx
+++ b/30_output_share/04_컬럼계보매핑.xlsx
@@ -1944,12 +1944,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>컬럼확정(2단)</t>
+          <t>컬럼확정(동명통과)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>컬럼확정(2단)</t>
+          <t>컬럼확정(동명통과)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>컬럼확정(2단)</t>
+          <t>컬럼확정(동명통과)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -9802,12 +9802,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -10974,7 +10974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11062,7 +11062,11 @@
           <t>CRM_BIZ_TARGET.MONTH_KEY</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
@@ -11076,12 +11080,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>비영 1,260/1,260 (100%)</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11110,11 @@
           <t>CRM_BIZ_TARGET.MONTH_KEY</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
@@ -11120,12 +11128,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>비영 1,260/1,260 (100%)</t>
         </is>
       </c>
     </row>
@@ -11150,7 +11158,11 @@
           <t>CRM_BIZ_TARGET.MONTH_KEY</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
@@ -11164,12 +11176,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>비영 1,260/1,260 (100%)</t>
         </is>
       </c>
     </row>
@@ -11194,7 +11206,11 @@
           <t>CRM_BIZ_TARGET.TARGET_CNT</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
@@ -11208,12 +11224,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>비영 1,260/1,260 (100%)</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11254,11 @@
           <t>CRM_BIZ_TARGET.TARGET_CNT</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
@@ -11257,7 +11277,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>전건 NULL (0/1,260)</t>
         </is>
       </c>
     </row>
@@ -11282,7 +11302,11 @@
           <t>CRM_BIZ_TARGET.TARGET_CNT</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
@@ -11301,7 +11325,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>전건 NULL (0/1,260)</t>
         </is>
       </c>
     </row>
@@ -11326,7 +11350,11 @@
           <t>CRM_BIZ_TARGET.TARGET_CNT</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
@@ -11345,7 +11373,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>`FACT_TARGET_PROJECT` 0행 — 원천 미입고</t>
+          <t>전건 NULL (0/1,260)</t>
         </is>
       </c>
     </row>
@@ -11778,6 +11806,390 @@
       <c r="J17" t="inlineStr">
         <is>
           <t>비영 36,769/36,769 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>GOAL_TYPE_NM</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.GOAL_TYPE_NM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.GOAL_TYPE_NM</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>비영 1,260/1,260 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CPR_DIV_NM</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.CPR_DIV_NM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.CPR_DIV_NM</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>비영 1,260/1,260 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ORG_PATH</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>DIM_ORG.ORG_PATH</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CRM_ORG.USE_YN</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TM_CM_DEPT_INFO</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>비영 1,305/1,315 (99.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SRC_TEAM_NM</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.SRC_TEAM_NM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.ORG_NM</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>비영 1,260/1,260 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SRC_SPONSOR_BIZ_NM</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.SRC_SPONSOR_BIZ_NM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.SPONSOR_BIZ_NM</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>비영 1,260/1,260 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>NEW_OLD_DIV_NM</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.NEW_OLD_DIV_NM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.NEW_OLD_DIV_NM</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>비영 820/1,260 (65.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ORG_DIV_NM</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.ORG_DIV_NM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.ORG_DIV_NM</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>비영 1,260/1,260 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>WIDE_TARGET_BIZ</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DTL_DIV_NM</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FACT_TARGET_PROJECT.DTL_DIV_NM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CRM_BIZ_TARGET.DTL_DIV_NM</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TM_CM_MBER_DVLP_GOAL_DIV</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>직접참조</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>컬럼확정</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>비영 338/1,260 (26.8%)</t>
         </is>
       </c>
     </row>
@@ -13510,12 +13922,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>비영 48,457/77,505 (62.5%)</t>
+          <t>비영 77,505/77,505 (100%)</t>
         </is>
       </c>
     </row>
@@ -17052,12 +17464,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -17249,7 +17661,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>비영 2/2 (100%)</t>
+          <t>비영 4/4 (100%)</t>
         </is>
       </c>
     </row>
@@ -18050,12 +18462,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -18727,7 +19139,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>비영 2/2 (100%)</t>
+          <t>비영 4/4 (100%)</t>
         </is>
       </c>
     </row>
@@ -18775,7 +19187,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>비영 2/2 (100%)</t>
+          <t>비영 4/4 (100%)</t>
         </is>
       </c>
     </row>
@@ -18896,12 +19308,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,663,437/1,663,437 (100%)</t>
         </is>
       </c>
     </row>
@@ -18944,12 +19356,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,663,437/1,663,437 (100%)</t>
         </is>
       </c>
     </row>
@@ -18992,12 +19404,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,663,437/1,663,437 (100%)</t>
         </is>
       </c>
     </row>
@@ -19040,12 +19452,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 98,168/1,663,437 (5.9%)</t>
         </is>
       </c>
     </row>
@@ -19088,12 +19500,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,663,437/1,663,437 (100%)</t>
         </is>
       </c>
     </row>
@@ -19136,12 +19548,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 452,903/1,663,437 (27.2%)</t>
         </is>
       </c>
     </row>
@@ -19184,12 +19596,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,663,437/1,663,437 (100%)</t>
         </is>
       </c>
     </row>
@@ -19232,12 +19644,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,545,982/1,663,437 (92.9%)</t>
         </is>
       </c>
     </row>
@@ -19280,12 +19692,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 330,438/1,663,437 (19.9%)</t>
         </is>
       </c>
     </row>
@@ -19328,12 +19740,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 995,447/1,663,437 (59.8%)</t>
         </is>
       </c>
     </row>
@@ -19376,12 +19788,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,663,437/1,663,437 (100%)</t>
         </is>
       </c>
     </row>
@@ -19429,7 +19841,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>전건 NULL (0/1,663,437)</t>
         </is>
       </c>
     </row>
@@ -19477,7 +19889,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>전건 NULL (0/1,663,437)</t>
         </is>
       </c>
     </row>
@@ -19520,12 +19932,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,545,982/1,663,437 (92.9%)</t>
         </is>
       </c>
     </row>
@@ -19568,12 +19980,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>`FACT_BIGQUERY_BEHAVIOR` 0행 — 원천 미입고</t>
+          <t>비영 1,529,725/1,663,437 (92.0%)</t>
         </is>
       </c>
     </row>
@@ -19808,12 +20220,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -20000,12 +20412,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,785,300)</t>
+          <t>비영 39,773/1,785,300 (2.2%)</t>
         </is>
       </c>
     </row>
@@ -20048,12 +20460,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>비영 1/1 (100%)</t>
+          <t>비영 47,858/47,859 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -20096,12 +20508,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>비영 1/1 (100%)</t>
+          <t>비영 47,842/47,859 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -20144,12 +20556,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>비영 1/1 (100%)</t>
+          <t>비영 47,856/47,859 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -20192,12 +20604,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>비영 1/1 (100%)</t>
+          <t>비영 469/480 (97.7%)</t>
         </is>
       </c>
     </row>
@@ -20240,12 +20652,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>비영 1/1 (100%)</t>
+          <t>비영 467/480 (97.3%)</t>
         </is>
       </c>
     </row>
@@ -20288,12 +20700,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1)</t>
+          <t>비영 479/480 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -20336,12 +20748,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1)</t>
+          <t>비영 479/480 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -20384,12 +20796,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1)</t>
+          <t>비영 479/480 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -20437,7 +20849,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>비영 2/2 (100%)</t>
+          <t>비영 4/4 (100%)</t>
         </is>
       </c>
     </row>
@@ -23276,12 +23688,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -26034,12 +26446,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/73,415) — 설계O·값 미주입</t>
+          <t>비영 251/73,415 (0.3%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
20261001_mstr 이관 가능성 테스트(PoC..)
</commit_message>
<xml_diff>
--- a/30_output_share/04_컬럼계보매핑.xlsx
+++ b/30_output_share/04_컬럼계보매핑.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>비영 48,457/48,457 (100%)</t>
+          <t>비영 50,096/50,096 (100%)</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 58,678/77,505 (75.7%)</t>
+          <t>비영 245,204/271,175 (90.4%)</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>비영 21,459/77,505 (27.7%)</t>
+          <t>비영 22,599/271,175 (8.3%)</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>비영 37,106/48,457 (76.6%)</t>
+          <t>비영 38,745/50,096 (77.3%)</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>비영 32,718/48,457 (67.5%)</t>
+          <t>비영 34,316/50,096 (68.5%)</t>
         </is>
       </c>
     </row>
@@ -885,7 +885,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>비영 2,104/48,457 (4.3%)</t>
+          <t>비영 2,104/50,096 (4.2%)</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>비영 33,721/48,457 (69.6%)</t>
+          <t>비영 35,319/50,096 (70.5%)</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>비영 15,993/48,457 (33.0%)</t>
+          <t>비영 17,591/50,096 (35.1%)</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>비영 45,121/48,457 (93.1%)</t>
+          <t>비영 46,760/50,096 (93.3%)</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>비영 36,009/48,457 (74.3%)</t>
+          <t>비영 37,607/50,096 (75.1%)</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>비영 48,457/48,457 (100%)</t>
+          <t>비영 50,096/50,096 (100%)</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>비영 42,618/48,457 (88.0%)</t>
+          <t>비영 44,586/50,096 (89.0%)</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>비영 14,990/48,457 (30.9%)</t>
+          <t>비영 16,588/50,096 (33.1%)</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>비영 32,933/48,457 (68.0%)</t>
+          <t>비영 35,539/50,096 (70.9%)</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>비영 35,002/48,457 (72.2%)</t>
+          <t>비영 36,641/50,096 (73.1%)</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>비영 32,902/48,457 (67.9%)</t>
+          <t>비영 34,500/50,096 (68.9%)</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>비영 45,974/48,457 (94.9%)</t>
+          <t>비영 47,992/50,096 (95.8%)</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>비영 2,104/48,457 (4.3%)</t>
+          <t>비영 2,104/50,096 (4.2%)</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>비영 35,943/48,457 (74.2%)</t>
+          <t>비영 37,541/50,096 (74.9%)</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>전건 NULL (0/48,457)</t>
+          <t>전건 NULL (0/50,096)</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>비영 7,953/48,457 (16.4%)</t>
+          <t>비영 7,953/50,096 (15.9%)</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>비영 7,953/48,457 (16.4%)</t>
+          <t>비영 7,953/50,096 (15.9%)</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>비영 13,971/48,457 (28.8%)</t>
+          <t>비영 14,795/50,096 (29.5%)</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>비영 17,801/48,457 (36.7%)</t>
+          <t>비영 18,832/50,096 (37.6%)</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>비영 3,366/3,367 (100.0%)</t>
+          <t>비영 9,679/9,696 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>비영 3,357/3,367 (99.7%)</t>
+          <t>비영 9,686/9,696 (99.9%)</t>
         </is>
       </c>
     </row>
@@ -8581,12 +8581,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -8597,7 +8597,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>비영 52,657/41,935,344 (0.1%)</t>
+          <t>비영 50,401/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8629,12 +8629,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -8645,7 +8645,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>비영 52,407/41,935,344 (0.1%)</t>
+          <t>비영 50,173/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8677,12 +8677,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -8693,7 +8693,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>비영 34,332/41,935,344 (0.1%)</t>
+          <t>비영 34,059/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8725,12 +8725,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -8741,7 +8741,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>비영 34,106/41,935,344 (0.1%)</t>
+          <t>비영 33,882/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8773,12 +8773,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -8789,7 +8789,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>비영 30,696/41,935,344 (0.1%)</t>
+          <t>비영 26,873/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8821,12 +8821,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>비영 30,187/41,935,344 (0.1%)</t>
+          <t>비영 26,416/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8869,12 +8869,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>비영 157,097/41,935,344 (0.4%)</t>
+          <t>비영 111,268/41,935,344 (0.3%)</t>
         </is>
       </c>
     </row>
@@ -8917,12 +8917,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>비영 70,027/41,935,344 (0.2%)</t>
+          <t>비영 34,342/41,935,344 (0.1%)</t>
         </is>
       </c>
     </row>
@@ -8965,12 +8965,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CRM_RELATION_ACTIVITY;CRM_SEND_MEMBER;CRM_SEND_REQUEST;CRM_SPONSOR_RELATION</t>
+          <t>CRM_SEND_REQUEST.TIT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;SND_REQ_MST;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL;TM_MM_FDRM_MBER_SPNSR_BSNS;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG;TM_RM_RELATNSP_GFTMNEY_INFO;TM_RM_RELATNSP_LETTER_INFO;TM_RM_RELATNSP_MSTR_INFO</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -8981,7 +8981,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>테이블수준</t>
+          <t>컬럼확정</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -9157,12 +9157,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CRM_SEND_MEMBER.SNDNG_RST_CD</t>
+          <t>CRM_SEND_REQUEST.SEND_STATUS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SND_MEMBER_LIST;SND_MEMBER_OPEN_LOG;TC_CMMN_DTL_CD;TD_MS_EMAIL_SNDNG_DTLS;TD_MS_MSG_AT_SNDNG_DTLS;TD_MS_PSTMTR_SNDNG_DTL</t>
+          <t>SND_REQ_MST;TM_MS_EMAIL_SNDNG;TM_MS_MSG_AT_SNDNG;TM_MS_PSTMTR_SNDNG</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -11085,7 +11085,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,966/2,966 (100%)</t>
         </is>
       </c>
     </row>
@@ -11133,7 +11133,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,966/2,966 (100%)</t>
         </is>
       </c>
     </row>
@@ -11181,7 +11181,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,966/2,966 (100%)</t>
         </is>
       </c>
     </row>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,966/2,966 (100%)</t>
         </is>
       </c>
     </row>
@@ -11277,7 +11277,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,260)</t>
+          <t>전건 NULL (0/2,966)</t>
         </is>
       </c>
     </row>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,260)</t>
+          <t>전건 NULL (0/2,966)</t>
         </is>
       </c>
     </row>
@@ -11373,7 +11373,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,260)</t>
+          <t>전건 NULL (0/2,966)</t>
         </is>
       </c>
     </row>
@@ -11853,7 +11853,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,966/2,966 (100%)</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,966/2,966 (100%)</t>
         </is>
       </c>
     </row>
@@ -11992,12 +11992,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 1,260/2,966 (42.5%)</t>
         </is>
       </c>
     </row>
@@ -12040,12 +12040,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 2,786/2,966 (93.9%)</t>
         </is>
       </c>
     </row>
@@ -12093,7 +12093,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>비영 820/1,260 (65.1%)</t>
+          <t>비영 2,526/2,966 (85.2%)</t>
         </is>
       </c>
     </row>
@@ -12136,12 +12136,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>비영 1,260/1,260 (100%)</t>
+          <t>비영 1,804/2,966 (60.8%)</t>
         </is>
       </c>
     </row>
@@ -12189,7 +12189,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>비영 338/1,260 (26.8%)</t>
+          <t>비영 440/2,966 (14.8%)</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -12969,7 +12969,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -13209,7 +13209,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>비영 2,104/48,457 (4.3%)</t>
+          <t>비영 2,104/50,096 (4.2%)</t>
         </is>
       </c>
     </row>
@@ -13257,7 +13257,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>비영 36,009/48,457 (74.3%)</t>
+          <t>비영 37,607/50,096 (75.1%)</t>
         </is>
       </c>
     </row>
@@ -13305,7 +13305,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>비영 48,457/48,457 (100%)</t>
+          <t>비영 50,096/50,096 (100%)</t>
         </is>
       </c>
     </row>
@@ -13353,7 +13353,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>비영 45,121/48,457 (93.1%)</t>
+          <t>비영 46,760/50,096 (93.3%)</t>
         </is>
       </c>
     </row>
@@ -13687,7 +13687,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -13735,7 +13735,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -13783,7 +13783,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/77,505) — 설계O·값 미주입</t>
+          <t>전건 0 (비영 0/271,175) — 설계O·값 미주입</t>
         </is>
       </c>
     </row>
@@ -13831,7 +13831,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 19,952/77,505 (25.7%)</t>
+          <t>비영 151,450/271,175 (55.8%)</t>
         </is>
       </c>
     </row>
@@ -13879,7 +13879,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>전건 0 (비영 0/77,505) — 설계O·값 미주입</t>
+          <t>전건 0 (비영 0/271,175) — 설계O·값 미주입</t>
         </is>
       </c>
     </row>
@@ -13927,7 +13927,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -13975,7 +13975,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>비영 58,678/77,505 (75.7%)</t>
+          <t>비영 245,204/271,175 (90.4%)</t>
         </is>
       </c>
     </row>
@@ -14023,7 +14023,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>비영 23,255/77,505 (30.0%)</t>
+          <t>비영 210,773/271,175 (77.7%)</t>
         </is>
       </c>
     </row>
@@ -14071,7 +14071,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>비영 25,148/77,505 (32.4%)</t>
+          <t>비영 189,300/271,175 (69.8%)</t>
         </is>
       </c>
     </row>
@@ -14119,7 +14119,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>비영 21,459/77,505 (27.7%)</t>
+          <t>비영 22,599/271,175 (8.3%)</t>
         </is>
       </c>
     </row>
@@ -14167,7 +14167,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>비영 7,139/77,505 (9.2%)</t>
+          <t>비영 50,949/271,175 (18.8%)</t>
         </is>
       </c>
     </row>
@@ -14215,7 +14215,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>비영 7,139/77,505 (9.2%)</t>
+          <t>비영 50,948/271,175 (18.8%)</t>
         </is>
       </c>
     </row>
@@ -14263,7 +14263,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -14311,7 +14311,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -14407,7 +14407,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>비영 1,025/29,048 (3.5%)</t>
+          <t>비영 1,033/221,079 (0.5%)</t>
         </is>
       </c>
     </row>
@@ -14455,7 +14455,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>비영 2,904/29,048 (10.0%)</t>
+          <t>비영 2,927/221,079 (1.3%)</t>
         </is>
       </c>
     </row>
@@ -14503,7 +14503,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>전건 NULL (0/29,048)</t>
+          <t>전건 NULL (0/221,079)</t>
         </is>
       </c>
     </row>
@@ -14546,12 +14546,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>비영 29,048/29,048 (100%)</t>
+          <t>비영 105,384/221,079 (47.7%)</t>
         </is>
       </c>
     </row>
@@ -14599,7 +14599,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>비영 29,048/29,048 (100%)</t>
+          <t>비영 221,079/221,079 (100%)</t>
         </is>
       </c>
     </row>
@@ -14647,7 +14647,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>비영 6,392/29,048 (22.0%)</t>
+          <t>비영 6,392/221,079 (2.9%)</t>
         </is>
       </c>
     </row>
@@ -14695,7 +14695,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>전건 NULL (0/29,048)</t>
+          <t>전건 NULL (0/221,079)</t>
         </is>
       </c>
     </row>
@@ -14743,7 +14743,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>전건 NULL (0/29,048)</t>
+          <t>전건 NULL (0/221,079)</t>
         </is>
       </c>
     </row>
@@ -14791,7 +14791,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>비영 15,893/29,048 (54.7%)</t>
+          <t>비영 17,738/221,079 (8.0%)</t>
         </is>
       </c>
     </row>
@@ -14839,7 +14839,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>비영 4,226/29,048 (14.5%)</t>
+          <t>비영 4,767/221,079 (2.2%)</t>
         </is>
       </c>
     </row>
@@ -14887,7 +14887,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>비영 18,563/29,048 (63.9%)</t>
+          <t>비영 178,990/221,079 (81.0%)</t>
         </is>
       </c>
     </row>
@@ -14935,7 +14935,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>비영 20,064/29,048 (69.1%)</t>
+          <t>비영 201,795/221,079 (91.3%)</t>
         </is>
       </c>
     </row>
@@ -14983,7 +14983,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>비영 6,226/29,048 (21.4%)</t>
+          <t>비영 49,087/221,079 (22.2%)</t>
         </is>
       </c>
     </row>
@@ -15031,7 +15031,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>비영 6,226/29,048 (21.4%)</t>
+          <t>비영 49,085/221,079 (22.2%)</t>
         </is>
       </c>
     </row>
@@ -15079,7 +15079,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>비영 6,392/29,048 (22.0%)</t>
+          <t>비영 6,392/221,079 (2.9%)</t>
         </is>
       </c>
     </row>
@@ -15127,7 +15127,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>비영 37,106/48,457 (76.6%)</t>
+          <t>비영 38,745/50,096 (77.3%)</t>
         </is>
       </c>
     </row>
@@ -15175,7 +15175,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>비영 32,718/48,457 (67.5%)</t>
+          <t>비영 34,316/50,096 (68.5%)</t>
         </is>
       </c>
     </row>
@@ -15223,7 +15223,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>비영 2,104/48,457 (4.3%)</t>
+          <t>비영 2,104/50,096 (4.2%)</t>
         </is>
       </c>
     </row>
@@ -15271,7 +15271,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>비영 33,721/48,457 (69.6%)</t>
+          <t>비영 35,319/50,096 (70.5%)</t>
         </is>
       </c>
     </row>
@@ -15319,7 +15319,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>비영 15,993/48,457 (33.0%)</t>
+          <t>비영 17,591/50,096 (35.1%)</t>
         </is>
       </c>
     </row>
@@ -15367,7 +15367,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>비영 45,121/48,457 (93.1%)</t>
+          <t>비영 46,760/50,096 (93.3%)</t>
         </is>
       </c>
     </row>
@@ -15415,7 +15415,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>비영 36,009/48,457 (74.3%)</t>
+          <t>비영 37,607/50,096 (75.1%)</t>
         </is>
       </c>
     </row>
@@ -15463,7 +15463,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>비영 48,457/48,457 (100%)</t>
+          <t>비영 50,096/50,096 (100%)</t>
         </is>
       </c>
     </row>
@@ -15511,7 +15511,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>비영 42,618/48,457 (88.0%)</t>
+          <t>비영 44,586/50,096 (89.0%)</t>
         </is>
       </c>
     </row>
@@ -15559,7 +15559,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>비영 14,990/48,457 (30.9%)</t>
+          <t>비영 16,588/50,096 (33.1%)</t>
         </is>
       </c>
     </row>
@@ -15607,7 +15607,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>비영 32,933/48,457 (68.0%)</t>
+          <t>비영 35,539/50,096 (70.9%)</t>
         </is>
       </c>
     </row>
@@ -15655,7 +15655,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>비영 35,002/48,457 (72.2%)</t>
+          <t>비영 36,641/50,096 (73.1%)</t>
         </is>
       </c>
     </row>
@@ -15703,7 +15703,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>비영 32,902/48,457 (67.9%)</t>
+          <t>비영 34,500/50,096 (68.9%)</t>
         </is>
       </c>
     </row>
@@ -15751,7 +15751,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>비영 45,974/48,457 (94.9%)</t>
+          <t>비영 47,992/50,096 (95.8%)</t>
         </is>
       </c>
     </row>
@@ -15799,7 +15799,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>비영 2,104/48,457 (4.3%)</t>
+          <t>비영 2,104/50,096 (4.2%)</t>
         </is>
       </c>
     </row>
@@ -15847,7 +15847,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>비영 35,943/48,457 (74.2%)</t>
+          <t>비영 37,541/50,096 (74.9%)</t>
         </is>
       </c>
     </row>
@@ -15895,7 +15895,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>전건 NULL (0/48,457)</t>
+          <t>전건 NULL (0/50,096)</t>
         </is>
       </c>
     </row>
@@ -15943,7 +15943,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>비영 7,953/48,457 (16.4%)</t>
+          <t>비영 7,953/50,096 (15.9%)</t>
         </is>
       </c>
     </row>
@@ -15991,7 +15991,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>비영 7,953/48,457 (16.4%)</t>
+          <t>비영 7,953/50,096 (15.9%)</t>
         </is>
       </c>
     </row>
@@ -16039,7 +16039,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>비영 13,971/48,457 (28.8%)</t>
+          <t>비영 14,795/50,096 (29.5%)</t>
         </is>
       </c>
     </row>
@@ -16087,7 +16087,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>비영 17,801/48,457 (36.7%)</t>
+          <t>비영 18,832/50,096 (37.6%)</t>
         </is>
       </c>
     </row>
@@ -16213,7 +16213,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>비영 29,048/29,048 (100%)</t>
+          <t>비영 221,079/221,079 (100%)</t>
         </is>
       </c>
     </row>
@@ -16261,7 +16261,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -16309,7 +16309,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -16357,7 +16357,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 58,678/77,505 (75.7%)</t>
+          <t>비영 245,204/271,175 (90.4%)</t>
         </is>
       </c>
     </row>
@@ -16405,7 +16405,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>비영 23,255/77,505 (30.0%)</t>
+          <t>비영 210,773/271,175 (77.7%)</t>
         </is>
       </c>
     </row>
@@ -16453,7 +16453,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>비영 25,148/77,505 (32.4%)</t>
+          <t>비영 189,300/271,175 (69.8%)</t>
         </is>
       </c>
     </row>
@@ -16501,7 +16501,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>비영 7,139/77,505 (9.2%)</t>
+          <t>비영 50,949/271,175 (18.8%)</t>
         </is>
       </c>
     </row>
@@ -16549,7 +16549,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>비영 7,139/77,505 (9.2%)</t>
+          <t>비영 50,948/271,175 (18.8%)</t>
         </is>
       </c>
     </row>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>비영 1,025/29,048 (3.5%)</t>
+          <t>비영 1,033/221,079 (0.5%)</t>
         </is>
       </c>
     </row>
@@ -16645,7 +16645,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>비영 2,904/29,048 (10.0%)</t>
+          <t>비영 2,927/221,079 (1.3%)</t>
         </is>
       </c>
     </row>
@@ -16693,7 +16693,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>전건 NULL (0/29,048)</t>
+          <t>전건 NULL (0/221,079)</t>
         </is>
       </c>
     </row>
@@ -16736,12 +16736,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>비영 29,048/29,048 (100%)</t>
+          <t>비영 105,384/221,079 (47.7%)</t>
         </is>
       </c>
     </row>
@@ -16789,7 +16789,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>비영 29,048/29,048 (100%)</t>
+          <t>비영 221,079/221,079 (100%)</t>
         </is>
       </c>
     </row>
@@ -16837,7 +16837,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>비영 6,392/29,048 (22.0%)</t>
+          <t>비영 6,392/221,079 (2.9%)</t>
         </is>
       </c>
     </row>
@@ -16885,7 +16885,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>전건 NULL (0/29,048)</t>
+          <t>전건 NULL (0/221,079)</t>
         </is>
       </c>
     </row>
@@ -16933,7 +16933,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>전건 NULL (0/29,048)</t>
+          <t>전건 NULL (0/221,079)</t>
         </is>
       </c>
     </row>
@@ -16981,7 +16981,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>비영 15,893/29,048 (54.7%)</t>
+          <t>비영 17,738/221,079 (8.0%)</t>
         </is>
       </c>
     </row>
@@ -17029,7 +17029,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>비영 4,226/29,048 (14.5%)</t>
+          <t>비영 4,767/221,079 (2.2%)</t>
         </is>
       </c>
     </row>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>비영 18,563/29,048 (63.9%)</t>
+          <t>비영 178,990/221,079 (81.0%)</t>
         </is>
       </c>
     </row>
@@ -17125,7 +17125,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>비영 20,064/29,048 (69.1%)</t>
+          <t>비영 201,795/221,079 (91.3%)</t>
         </is>
       </c>
     </row>
@@ -17173,7 +17173,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>비영 6,226/29,048 (21.4%)</t>
+          <t>비영 49,087/221,079 (22.2%)</t>
         </is>
       </c>
     </row>
@@ -17221,7 +17221,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>비영 6,226/29,048 (21.4%)</t>
+          <t>비영 49,085/221,079 (22.2%)</t>
         </is>
       </c>
     </row>
@@ -17269,7 +17269,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>비영 6,392/29,048 (22.0%)</t>
+          <t>비영 6,392/221,079 (2.9%)</t>
         </is>
       </c>
     </row>
@@ -17565,7 +17565,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>비영 3,366/3,367 (100.0%)</t>
+          <t>비영 9,679/9,696 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -17613,7 +17613,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>비영 3,357/3,367 (99.7%)</t>
+          <t>비영 9,686/9,696 (99.9%)</t>
         </is>
       </c>
     </row>
@@ -17787,7 +17787,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -17835,7 +17835,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -17883,7 +17883,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>비영 58,678/77,505 (75.7%)</t>
+          <t>비영 245,204/271,175 (90.4%)</t>
         </is>
       </c>
     </row>
@@ -17931,7 +17931,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 23,255/77,505 (30.0%)</t>
+          <t>비영 210,773/271,175 (77.7%)</t>
         </is>
       </c>
     </row>
@@ -17979,7 +17979,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>비영 25,148/77,505 (32.4%)</t>
+          <t>비영 189,300/271,175 (69.8%)</t>
         </is>
       </c>
     </row>
@@ -18027,7 +18027,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>비영 21,459/77,505 (27.7%)</t>
+          <t>비영 22,599/271,175 (8.3%)</t>
         </is>
       </c>
     </row>
@@ -18075,7 +18075,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>비영 7,139/77,505 (9.2%)</t>
+          <t>비영 50,949/271,175 (18.8%)</t>
         </is>
       </c>
     </row>
@@ -18123,7 +18123,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>비영 7,139/77,505 (9.2%)</t>
+          <t>비영 50,948/271,175 (18.8%)</t>
         </is>
       </c>
     </row>
@@ -18171,7 +18171,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -18219,7 +18219,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -18267,7 +18267,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>비영 77,505/77,505 (100%)</t>
+          <t>비영 271,175/271,175 (100%)</t>
         </is>
       </c>
     </row>
@@ -18803,7 +18803,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>비영 3,367/3,367 (100%)</t>
+          <t>비영 9,696/9,696 (100%)</t>
         </is>
       </c>
     </row>
@@ -18851,7 +18851,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>비영 3,366/3,367 (100.0%)</t>
+          <t>비영 9,679/9,696 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -18899,7 +18899,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>비영 3,366/3,367 (100.0%)</t>
+          <t>비영 9,695/9,696 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -18947,7 +18947,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>전건 NULL (0/3,367)</t>
+          <t>전건 NULL (0/9,696)</t>
         </is>
       </c>
     </row>
@@ -18995,7 +18995,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>비영 3,357/3,367 (99.7%)</t>
+          <t>비영 9,686/9,696 (99.9%)</t>
         </is>
       </c>
     </row>
@@ -19043,7 +19043,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>비영 3,366/3,367 (100.0%)</t>
+          <t>비영 6,423/9,696 (66.2%)</t>
         </is>
       </c>
     </row>
@@ -19091,7 +19091,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>전건 NULL (0/3,367)</t>
+          <t>전건 NULL (0/9,696)</t>
         </is>
       </c>
     </row>
@@ -19313,7 +19313,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>비영 1,663,437/1,663,437 (100%)</t>
+          <t>비영 1,398,512/1,398,512 (100%)</t>
         </is>
       </c>
     </row>
@@ -19361,7 +19361,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>비영 1,663,437/1,663,437 (100%)</t>
+          <t>비영 1,398,512/1,398,512 (100%)</t>
         </is>
       </c>
     </row>
@@ -19409,7 +19409,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>비영 1,663,437/1,663,437 (100%)</t>
+          <t>비영 1,398,512/1,398,512 (100%)</t>
         </is>
       </c>
     </row>
@@ -19457,7 +19457,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>비영 98,168/1,663,437 (5.9%)</t>
+          <t>비영 80,624/1,398,512 (5.8%)</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>비영 1,663,437/1,663,437 (100%)</t>
+          <t>비영 1,398,512/1,398,512 (100%)</t>
         </is>
       </c>
     </row>
@@ -19553,7 +19553,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>비영 452,903/1,663,437 (27.2%)</t>
+          <t>비영 374,079/1,398,512 (26.7%)</t>
         </is>
       </c>
     </row>
@@ -19601,7 +19601,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>비영 1,663,437/1,663,437 (100%)</t>
+          <t>비영 1,398,512/1,398,512 (100%)</t>
         </is>
       </c>
     </row>
@@ -19649,7 +19649,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>비영 1,545,982/1,663,437 (92.9%)</t>
+          <t>비영 1,302,628/1,398,512 (93.1%)</t>
         </is>
       </c>
     </row>
@@ -19697,7 +19697,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>비영 330,438/1,663,437 (19.9%)</t>
+          <t>비영 294,660/1,398,512 (21.1%)</t>
         </is>
       </c>
     </row>
@@ -19745,7 +19745,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>비영 995,447/1,663,437 (59.8%)</t>
+          <t>비영 1,003,028/1,398,512 (71.7%)</t>
         </is>
       </c>
     </row>
@@ -19793,7 +19793,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>비영 1,663,437/1,663,437 (100%)</t>
+          <t>비영 1,398,512/1,398,512 (100%)</t>
         </is>
       </c>
     </row>
@@ -19841,7 +19841,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,663,437)</t>
+          <t>전건 NULL (0/1,398,512)</t>
         </is>
       </c>
     </row>
@@ -19889,7 +19889,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,663,437)</t>
+          <t>전건 NULL (0/1,398,512)</t>
         </is>
       </c>
     </row>
@@ -19937,7 +19937,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>비영 1,545,982/1,663,437 (92.9%)</t>
+          <t>비영 1,302,628/1,398,512 (93.1%)</t>
         </is>
       </c>
     </row>
@@ -19985,7 +19985,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>비영 1,529,725/1,663,437 (92.0%)</t>
+          <t>비영 1,282,053/1,398,512 (91.7%)</t>
         </is>
       </c>
     </row>
@@ -20417,7 +20417,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>비영 39,773/1,785,300 (2.2%)</t>
+          <t>비영 30,397/1,785,300 (1.7%)</t>
         </is>
       </c>
     </row>
@@ -20465,7 +20465,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>비영 47,858/47,859 (100.0%)</t>
+          <t>비영 41,761/41,762 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -20513,7 +20513,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>비영 47,842/47,859 (100.0%)</t>
+          <t>비영 41,745/41,762 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -20561,7 +20561,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>비영 47,856/47,859 (100.0%)</t>
+          <t>비영 41,759/41,762 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -20609,7 +20609,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>비영 469/480 (97.7%)</t>
+          <t>비영 521/533 (97.7%)</t>
         </is>
       </c>
     </row>
@@ -20657,7 +20657,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>비영 467/480 (97.3%)</t>
+          <t>비영 518/533 (97.2%)</t>
         </is>
       </c>
     </row>
@@ -20705,7 +20705,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>비영 479/480 (99.8%)</t>
+          <t>비영 532/533 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -20753,7 +20753,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>비영 479/480 (99.8%)</t>
+          <t>비영 532/533 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -20801,7 +20801,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>비영 479/480 (99.8%)</t>
+          <t>비영 532/533 (99.8%)</t>
         </is>
       </c>
     </row>
@@ -22803,7 +22803,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CRM_EVENT_PARTICIPATION.PRZWIN_CD</t>
+          <t>CRM_EVENT_PARTICIPATION.SELF_PARTCPT_CD</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -22824,12 +22824,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>WAIT</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>전건 NULL (0/1,248,727)</t>
+          <t>비영 162,441/1,248,727 (13.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>